<commit_message>
add category-based person pool rotation
</commit_message>
<xml_diff>
--- a/products/商品信息表.xlsx
+++ b/products/商品信息表.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品信息" sheetId="1" r:id="Rca19d8f72c1a4555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R91e9602462b741bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品信息" sheetId="1" r:id="R821728b4b4e14592"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Raadc62020779476d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -259,15 +259,17 @@
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="32" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="32" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="32" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -281,30 +283,36 @@
         <x:v>selling_points</x:v>
       </x:c>
       <x:c r="D1" s="2" t="str">
+        <x:v>category</x:v>
+      </x:c>
+      <x:c r="E1" s="2" t="str">
         <x:v>image_path</x:v>
       </x:c>
-      <x:c r="E1" s="2" t="str">
+      <x:c r="F1" s="2" t="str">
+        <x:v>person_image_path</x:v>
+      </x:c>
+      <x:c r="G1" s="2" t="str">
         <x:v>script</x:v>
       </x:c>
-      <x:c r="F1" s="2" t="str">
+      <x:c r="H1" s="2" t="str">
         <x:v>avatar</x:v>
       </x:c>
-      <x:c r="G1" s="2" t="str">
+      <x:c r="I1" s="2" t="str">
         <x:v>voice</x:v>
       </x:c>
-      <x:c r="H1" s="2" t="str">
+      <x:c r="J1" s="2" t="str">
         <x:v>duration_seconds</x:v>
       </x:c>
-      <x:c r="I1" s="2" t="str">
+      <x:c r="K1" s="2" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="J1" s="2" t="str">
+      <x:c r="L1" s="2" t="str">
         <x:v>retry_count</x:v>
       </x:c>
-      <x:c r="K1" s="2" t="str">
+      <x:c r="M1" s="2" t="str">
         <x:v>output_path</x:v>
       </x:c>
-      <x:c r="L1" s="2" t="str">
+      <x:c r="N1" s="2" t="str">
         <x:v>error_message</x:v>
       </x:c>
     </x:row>
@@ -319,24 +327,28 @@
         <x:v>根系完整；叶片厚实；清炒清甜</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
+        <x:v>fresh_food</x:v>
+      </x:c>
+      <x:c r="E2" s="5" t="str">
         <x:v>products/images/SKU001.png</x:v>
       </x:c>
-      <x:c r="E2" s="5" t="str">
+      <x:c r="F2" s="5" t="str"/>
+      <x:c r="G2" s="5" t="str">
         <x:v>最近买菜最怕不新鲜？这个小青菜我真的会回购。根系完整，叶片厚实，清炒也很嫩。</x:v>
       </x:c>
-      <x:c r="F2" s="5" t="str"/>
-      <x:c r="G2" s="5" t="str"/>
-      <x:c r="H2" s="5" t="n">
+      <x:c r="H2" s="5" t="str"/>
+      <x:c r="I2" s="5" t="str"/>
+      <x:c r="J2" s="5" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="I2" s="5" t="str">
+      <x:c r="K2" s="5" t="str">
         <x:v>pending</x:v>
       </x:c>
-      <x:c r="J2" s="5" t="n">
+      <x:c r="L2" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K2" s="5" t="str"/>
-      <x:c r="L2" s="5" t="str"/>
+      <x:c r="M2" s="5" t="str"/>
+      <x:c r="N2" s="5" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5"/>
@@ -351,6 +363,8 @@
       <x:c r="J3" s="5"/>
       <x:c r="K3" s="5"/>
       <x:c r="L3" s="5"/>
+      <x:c r="M3" s="5"/>
+      <x:c r="N3" s="5"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="5"/>
@@ -365,6 +379,8 @@
       <x:c r="J4" s="5"/>
       <x:c r="K4" s="5"/>
       <x:c r="L4" s="5"/>
+      <x:c r="M4" s="5"/>
+      <x:c r="N4" s="5"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="5"/>
@@ -379,6 +395,8 @@
       <x:c r="J5" s="5"/>
       <x:c r="K5" s="5"/>
       <x:c r="L5" s="5"/>
+      <x:c r="M5" s="5"/>
+      <x:c r="N5" s="5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="5"/>
@@ -393,6 +411,8 @@
       <x:c r="J6" s="5"/>
       <x:c r="K6" s="5"/>
       <x:c r="L6" s="5"/>
+      <x:c r="M6" s="5"/>
+      <x:c r="N6" s="5"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="5"/>
@@ -407,6 +427,8 @@
       <x:c r="J7" s="5"/>
       <x:c r="K7" s="5"/>
       <x:c r="L7" s="5"/>
+      <x:c r="M7" s="5"/>
+      <x:c r="N7" s="5"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="5"/>
@@ -421,6 +443,8 @@
       <x:c r="J8" s="5"/>
       <x:c r="K8" s="5"/>
       <x:c r="L8" s="5"/>
+      <x:c r="M8" s="5"/>
+      <x:c r="N8" s="5"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="5"/>
@@ -435,6 +459,8 @@
       <x:c r="J9" s="5"/>
       <x:c r="K9" s="5"/>
       <x:c r="L9" s="5"/>
+      <x:c r="M9" s="5"/>
+      <x:c r="N9" s="5"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="5"/>
@@ -449,6 +475,8 @@
       <x:c r="J10" s="5"/>
       <x:c r="K10" s="5"/>
       <x:c r="L10" s="5"/>
+      <x:c r="M10" s="5"/>
+      <x:c r="N10" s="5"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5"/>
@@ -463,6 +491,8 @@
       <x:c r="J11" s="5"/>
       <x:c r="K11" s="5"/>
       <x:c r="L11" s="5"/>
+      <x:c r="M11" s="5"/>
+      <x:c r="N11" s="5"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="5"/>
@@ -477,6 +507,8 @@
       <x:c r="J12" s="5"/>
       <x:c r="K12" s="5"/>
       <x:c r="L12" s="5"/>
+      <x:c r="M12" s="5"/>
+      <x:c r="N12" s="5"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="5"/>
@@ -491,6 +523,8 @@
       <x:c r="J13" s="5"/>
       <x:c r="K13" s="5"/>
       <x:c r="L13" s="5"/>
+      <x:c r="M13" s="5"/>
+      <x:c r="N13" s="5"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="5"/>
@@ -505,6 +539,8 @@
       <x:c r="J14" s="5"/>
       <x:c r="K14" s="5"/>
       <x:c r="L14" s="5"/>
+      <x:c r="M14" s="5"/>
+      <x:c r="N14" s="5"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="5"/>
@@ -519,6 +555,8 @@
       <x:c r="J15" s="5"/>
       <x:c r="K15" s="5"/>
       <x:c r="L15" s="5"/>
+      <x:c r="M15" s="5"/>
+      <x:c r="N15" s="5"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="5"/>
@@ -533,6 +571,8 @@
       <x:c r="J16" s="5"/>
       <x:c r="K16" s="5"/>
       <x:c r="L16" s="5"/>
+      <x:c r="M16" s="5"/>
+      <x:c r="N16" s="5"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="5"/>
@@ -547,6 +587,8 @@
       <x:c r="J17" s="5"/>
       <x:c r="K17" s="5"/>
       <x:c r="L17" s="5"/>
+      <x:c r="M17" s="5"/>
+      <x:c r="N17" s="5"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="5"/>
@@ -561,6 +603,8 @@
       <x:c r="J18" s="5"/>
       <x:c r="K18" s="5"/>
       <x:c r="L18" s="5"/>
+      <x:c r="M18" s="5"/>
+      <x:c r="N18" s="5"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="5"/>
@@ -575,6 +619,8 @@
       <x:c r="J19" s="5"/>
       <x:c r="K19" s="5"/>
       <x:c r="L19" s="5"/>
+      <x:c r="M19" s="5"/>
+      <x:c r="N19" s="5"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="5"/>
@@ -589,6 +635,8 @@
       <x:c r="J20" s="5"/>
       <x:c r="K20" s="5"/>
       <x:c r="L20" s="5"/>
+      <x:c r="M20" s="5"/>
+      <x:c r="N20" s="5"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="5"/>
@@ -603,6 +651,8 @@
       <x:c r="J21" s="5"/>
       <x:c r="K21" s="5"/>
       <x:c r="L21" s="5"/>
+      <x:c r="M21" s="5"/>
+      <x:c r="N21" s="5"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="5"/>
@@ -617,6 +667,8 @@
       <x:c r="J22" s="5"/>
       <x:c r="K22" s="5"/>
       <x:c r="L22" s="5"/>
+      <x:c r="M22" s="5"/>
+      <x:c r="N22" s="5"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="5"/>
@@ -631,6 +683,8 @@
       <x:c r="J23" s="5"/>
       <x:c r="K23" s="5"/>
       <x:c r="L23" s="5"/>
+      <x:c r="M23" s="5"/>
+      <x:c r="N23" s="5"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="5"/>
@@ -645,6 +699,8 @@
       <x:c r="J24" s="5"/>
       <x:c r="K24" s="5"/>
       <x:c r="L24" s="5"/>
+      <x:c r="M24" s="5"/>
+      <x:c r="N24" s="5"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="5"/>
@@ -659,6 +715,8 @@
       <x:c r="J25" s="5"/>
       <x:c r="K25" s="5"/>
       <x:c r="L25" s="5"/>
+      <x:c r="M25" s="5"/>
+      <x:c r="N25" s="5"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="5"/>
@@ -673,6 +731,8 @@
       <x:c r="J26" s="5"/>
       <x:c r="K26" s="5"/>
       <x:c r="L26" s="5"/>
+      <x:c r="M26" s="5"/>
+      <x:c r="N26" s="5"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="5"/>
@@ -687,6 +747,8 @@
       <x:c r="J27" s="5"/>
       <x:c r="K27" s="5"/>
       <x:c r="L27" s="5"/>
+      <x:c r="M27" s="5"/>
+      <x:c r="N27" s="5"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="5"/>
@@ -701,6 +763,8 @@
       <x:c r="J28" s="5"/>
       <x:c r="K28" s="5"/>
       <x:c r="L28" s="5"/>
+      <x:c r="M28" s="5"/>
+      <x:c r="N28" s="5"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="5"/>
@@ -715,6 +779,8 @@
       <x:c r="J29" s="5"/>
       <x:c r="K29" s="5"/>
       <x:c r="L29" s="5"/>
+      <x:c r="M29" s="5"/>
+      <x:c r="N29" s="5"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="5"/>
@@ -729,6 +795,8 @@
       <x:c r="J30" s="5"/>
       <x:c r="K30" s="5"/>
       <x:c r="L30" s="5"/>
+      <x:c r="M30" s="5"/>
+      <x:c r="N30" s="5"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="5"/>
@@ -743,6 +811,8 @@
       <x:c r="J31" s="5"/>
       <x:c r="K31" s="5"/>
       <x:c r="L31" s="5"/>
+      <x:c r="M31" s="5"/>
+      <x:c r="N31" s="5"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="5"/>
@@ -757,6 +827,8 @@
       <x:c r="J32" s="5"/>
       <x:c r="K32" s="5"/>
       <x:c r="L32" s="5"/>
+      <x:c r="M32" s="5"/>
+      <x:c r="N32" s="5"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="5"/>
@@ -771,6 +843,8 @@
       <x:c r="J33" s="5"/>
       <x:c r="K33" s="5"/>
       <x:c r="L33" s="5"/>
+      <x:c r="M33" s="5"/>
+      <x:c r="N33" s="5"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="5"/>
@@ -785,6 +859,8 @@
       <x:c r="J34" s="5"/>
       <x:c r="K34" s="5"/>
       <x:c r="L34" s="5"/>
+      <x:c r="M34" s="5"/>
+      <x:c r="N34" s="5"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="5"/>
@@ -799,6 +875,8 @@
       <x:c r="J35" s="5"/>
       <x:c r="K35" s="5"/>
       <x:c r="L35" s="5"/>
+      <x:c r="M35" s="5"/>
+      <x:c r="N35" s="5"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="5"/>
@@ -813,6 +891,8 @@
       <x:c r="J36" s="5"/>
       <x:c r="K36" s="5"/>
       <x:c r="L36" s="5"/>
+      <x:c r="M36" s="5"/>
+      <x:c r="N36" s="5"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="5"/>
@@ -827,6 +907,8 @@
       <x:c r="J37" s="5"/>
       <x:c r="K37" s="5"/>
       <x:c r="L37" s="5"/>
+      <x:c r="M37" s="5"/>
+      <x:c r="N37" s="5"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="5"/>
@@ -841,6 +923,8 @@
       <x:c r="J38" s="5"/>
       <x:c r="K38" s="5"/>
       <x:c r="L38" s="5"/>
+      <x:c r="M38" s="5"/>
+      <x:c r="N38" s="5"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="5"/>
@@ -855,6 +939,8 @@
       <x:c r="J39" s="5"/>
       <x:c r="K39" s="5"/>
       <x:c r="L39" s="5"/>
+      <x:c r="M39" s="5"/>
+      <x:c r="N39" s="5"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="5"/>
@@ -869,6 +955,8 @@
       <x:c r="J40" s="5"/>
       <x:c r="K40" s="5"/>
       <x:c r="L40" s="5"/>
+      <x:c r="M40" s="5"/>
+      <x:c r="N40" s="5"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="5"/>
@@ -883,6 +971,8 @@
       <x:c r="J41" s="5"/>
       <x:c r="K41" s="5"/>
       <x:c r="L41" s="5"/>
+      <x:c r="M41" s="5"/>
+      <x:c r="N41" s="5"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="5"/>
@@ -897,6 +987,8 @@
       <x:c r="J42" s="5"/>
       <x:c r="K42" s="5"/>
       <x:c r="L42" s="5"/>
+      <x:c r="M42" s="5"/>
+      <x:c r="N42" s="5"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="5"/>
@@ -911,6 +1003,8 @@
       <x:c r="J43" s="5"/>
       <x:c r="K43" s="5"/>
       <x:c r="L43" s="5"/>
+      <x:c r="M43" s="5"/>
+      <x:c r="N43" s="5"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="5"/>
@@ -925,6 +1019,8 @@
       <x:c r="J44" s="5"/>
       <x:c r="K44" s="5"/>
       <x:c r="L44" s="5"/>
+      <x:c r="M44" s="5"/>
+      <x:c r="N44" s="5"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="5"/>
@@ -939,6 +1035,8 @@
       <x:c r="J45" s="5"/>
       <x:c r="K45" s="5"/>
       <x:c r="L45" s="5"/>
+      <x:c r="M45" s="5"/>
+      <x:c r="N45" s="5"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="5"/>
@@ -953,6 +1051,8 @@
       <x:c r="J46" s="5"/>
       <x:c r="K46" s="5"/>
       <x:c r="L46" s="5"/>
+      <x:c r="M46" s="5"/>
+      <x:c r="N46" s="5"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="5"/>
@@ -967,6 +1067,8 @@
       <x:c r="J47" s="5"/>
       <x:c r="K47" s="5"/>
       <x:c r="L47" s="5"/>
+      <x:c r="M47" s="5"/>
+      <x:c r="N47" s="5"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="5"/>
@@ -981,6 +1083,8 @@
       <x:c r="J48" s="5"/>
       <x:c r="K48" s="5"/>
       <x:c r="L48" s="5"/>
+      <x:c r="M48" s="5"/>
+      <x:c r="N48" s="5"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="5"/>
@@ -995,6 +1099,8 @@
       <x:c r="J49" s="5"/>
       <x:c r="K49" s="5"/>
       <x:c r="L49" s="5"/>
+      <x:c r="M49" s="5"/>
+      <x:c r="N49" s="5"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="5"/>
@@ -1009,10 +1115,12 @@
       <x:c r="J50" s="5"/>
       <x:c r="K50" s="5"/>
       <x:c r="L50" s="5"/>
+      <x:c r="M50" s="5"/>
+      <x:c r="N50" s="5"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="I2:I500">
+    <x:dataValidation type="list" sqref="K2:K500">
       <x:formula1>"pending,running,downloaded,failed,needs_review"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -1088,121 +1196,149 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>image_path</x:v>
+        <x:v>category</x:v>
       </x:c>
       <x:c r="B5" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>商品图片路径，建议放在 products/images/。</x:v>
+        <x:v>商品品类，用于从 assets/person_pool/&lt;category&gt;/ 自动轮换人物图。</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>products/images/SKU001.png</x:v>
+        <x:v>fresh_food</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>script</x:v>
+        <x:v>image_path</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>口播脚本；为空时后续由文案模块生成。</x:v>
+        <x:v>商品图片路径，建议放在 products/images/。</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>这个小青菜我真的会回购。</x:v>
+        <x:v>products/images/SKU001.png</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>avatar</x:v>
+        <x:v>person_image_path</x:v>
       </x:c>
       <x:c r="B7" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>飞影数字人配置，留空使用默认值。</x:v>
-      </x:c>
-      <x:c r="D7" t="str"/>
+        <x:v>指定人物图；留空时按 category 从人物池轮换，没有素材则按配置使用飞影推荐人物。</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>assets/person_pool/fresh_food/host_01.jpg</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>voice</x:v>
+        <x:v>script</x:v>
       </x:c>
       <x:c r="B8" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>声音配置，留空使用默认值。</x:v>
-      </x:c>
-      <x:c r="D8" t="str"/>
+        <x:v>口播脚本；为空时后续由文案模块生成。</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>这个小青菜我真的会回购。</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>duration_seconds</x:v>
+        <x:v>avatar</x:v>
       </x:c>
       <x:c r="B9" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>视频时长，建议 15-25 秒。</x:v>
-      </x:c>
-      <x:c r="D9" t="str">
-        <x:v>20</x:v>
-      </x:c>
+        <x:v>飞影数字人配置，留空使用默认值。</x:v>
+      </x:c>
+      <x:c r="D9" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>status</x:v>
+        <x:v>voice</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>任务状态，新任务填 pending。</x:v>
-      </x:c>
-      <x:c r="D10" t="str">
-        <x:v>pending</x:v>
-      </x:c>
+        <x:v>声音配置，留空使用默认值。</x:v>
+      </x:c>
+      <x:c r="D10" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>retry_count</x:v>
+        <x:v>duration_seconds</x:v>
       </x:c>
       <x:c r="B11" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>失败重试次数。</x:v>
+        <x:v>视频时长，建议 15-25 秒。</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>output_path</x:v>
+        <x:v>status</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>下载后的视频路径。</x:v>
-      </x:c>
-      <x:c r="D12" t="str"/>
+        <x:v>任务状态，新任务填 pending。</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>error_message</x:v>
+        <x:v>retry_count</x:v>
       </x:c>
       <x:c r="B13" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="C13" t="str">
+        <x:v>失败重试次数。</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>output_path</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>下载后的视频路径。</x:v>
+      </x:c>
+      <x:c r="D14" t="str"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>error_message</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
         <x:v>失败原因。</x:v>
       </x:c>
-      <x:c r="D13" t="str"/>
+      <x:c r="D15" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>